<commit_message>
fix v2 sprint 3
</commit_message>
<xml_diff>
--- a/reports/validation_report.xlsx
+++ b/reports/validation_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -688,6 +688,108 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Future Credits</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Future credits at OJT are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Future Failed Courses</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Future failed course values are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Future Missing Prerequisites</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Future missing prerequisite values are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Future Academic Warning</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Future academic warning values are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Future OJT Eligible</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Future OJT eligibility values are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>OJT Delay Outcome</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OJT delay outcomes are valid.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>